<commit_message>
Anomalies TVA : réponse recadrée sur les 3 reproches + réconciliation caisse/compta
Relit le grief exact (rapport p. 25-27 : bases négatives, somme TVA ≠ total,
non-correspondance avec la comptabilité) et reconstruit la page pour y répondre
point par point :
- distinction TVA réelle (tax_amount) vs champ « base HT » brut (résidu négatif)
- tableau de réconciliation : bases reconstituées = comptes 706300/706000 à
  quelques € près, alors que la base brute du fisc est aberrante et ne boucle
  pas au CA TTC
- mécanisme de la base 20 % négative (ticket multi-taux daté) + écart d'arrondi
  somme/total (0,01 %)
- écarts caisse/comptabilité chiffrés et expliqués (pourboire 706800, arrondis
  de retranscription manuelle), < 0,2 %, renvoi au grief suppressions
- onglet « Réconciliation caisse-compta » ajouté au XLSX

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/RF-anomalies-tva.xlsx
+++ b/public/documents/pieces-defense/RF-anomalies-tva.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Ventilation TVA par exercice" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Coherence par famille" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Ecarts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Reconciliation caisse-compta" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1092,4 +1093,244 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Exercice</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Base 10 % reconstituee (caisse)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Compta 706300</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ecart 10 %</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Base 20 % reconstituee (caisse)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Compta 706000</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Base 20 % brute (fisc)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>TVA caisse</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TVA compta 445710</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Ecart TVA</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CA TTC caisse</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CA TTC compta</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Ecart CA</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>dont pourboire 706800</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ex. clos 31/03/2023</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>296111</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>296105.87</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>5.130000000004657</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>64708.3</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>64712.51</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>-11645.01</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>42552.76</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>42614.45</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>-61.68999999999505</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>403370.42</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>404030.87</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>-660.4500000000116</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>598.04</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ex. clos 31/03/2024</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>319174.4</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>319179.31</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>-4.909999999974389</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>72413.2</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>72416.55</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>-1680.08</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>46400.08</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>46464.79</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>-64.70999999999913</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>437992.92</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>438658.43</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>-665.5100000000093</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>597.75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ex. clos 31/03/2025</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>318522</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>318345.43</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>176.570000000007</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>70372.14999999999</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>70517.47</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>572.55</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>45926.63</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>46005.45</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>-78.81999999999971</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>434827.86</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>435524.92</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>-697.0599999999977</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>656.5700000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Anomalies TVA : correction de l'exemple et parallèle fisc/défense
- Corrige une erreur factuelle : base brute du fichier pour la ligne 10 % du
  ticket n° 2 = 5,70 € (et non 14,30 €, qui est la base reconstituée).
- Remplace le mécanisme « résidu = TTC − base 10 % » (non vérifiable sur les
  données) par la preuve de non-additivité : 5,70 + (−14,80) = −9,10 € ≠ HT réel
  18,60 €. Ajout d'une ligne « Total ticket » au tableau d'exemple.
- Renforce l'anti-circularité : base = TVA/taux est l'inverse exact du calcul de
  TVA, validée par une source indépendante (compta manuscrite des Z).
- Ajoute un tableau comparatif « Méthode du service / Notre méthode » + le point
  décisif : le service utilise tax_amount pour la TVA p. 26 mais lit la base sur
  la colonne défectueuse.
- Régénère le XLSX (onglet exemple corrigé).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/RF-anomalies-tva.xlsx
+++ b/public/documents/pieces-defense/RF-anomalies-tva.xlsx
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>14.3</v>
+        <v>5.7</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>1.43</v>
@@ -1458,19 +1458,23 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TOTAL ticket</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
+          <t>TOTAL ticket (HT reel = 18,60 €)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>-9.1</v>
+      </c>
       <c r="C6" s="5" t="n">
         <v>2.3</v>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="5" t="n">
+        <v>18.65</v>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Lecture : le champ « base HT 20 % » de l'export vaut -14,80 € (residu non additif), mais la TVA reellement collectee au taux de 20 % est +0,87 € (base reelle 4,35 €). La TVA par ligne est toujours positive ; sa somme (1,43 + 0,87 = 2,30 €) egale la TVA totale du ticket. Effet sur la TVA et le CA : nul. Ce cas concerne 8526 lignes sur 29588 (28,8 %).</t>
+          <t>Lecture : les deux champs « base HT » bruts du fichier (5,70 € et -14,80 €) s'additionnent a -9,10 €, montant absurde pour une vente de 20,90 € (HT reel = 20,90 - 2,30 = 18,60 €) : la colonne « base » de l'export est non additive, donc non fiable. Les bases reconstituees base = TVA / taux (14,30 € + 4,35 €) redonnent 18,65 €, soit le HT reel a 5 centimes pres (arrondi de la TVA de chaque ligne). La TVA par ligne est toujours positive ; sa somme (1,43 + 0,87 = 2,30 €) egale la TVA totale du ticket. Effet sur la TVA et le CA : nul. Ce cas concerne 8526 lignes sur 29588 (28,8 %), toutes sur des tickets a deux taux.</t>
         </is>
       </c>
     </row>

</xml_diff>